<commit_message>
Final 2026 update after last matches
</commit_message>
<xml_diff>
--- a/output/2026_dorost.xlsx
+++ b/output/2026_dorost.xlsx
@@ -513,16 +513,16 @@
         </is>
       </c>
       <c r="C2" t="n">
+        <v>6</v>
+      </c>
+      <c r="D2" t="n">
         <v>5</v>
       </c>
-      <c r="D2" t="n">
-        <v>4</v>
-      </c>
       <c r="E2" t="n">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="F2" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="G2" t="n">
         <v>2</v>
@@ -531,13 +531,13 @@
         <v>1</v>
       </c>
       <c r="I2" s="2" t="n">
-        <v>0.5</v>
+        <v>0.4</v>
       </c>
       <c r="J2" t="n">
+        <v>8</v>
+      </c>
+      <c r="K2" t="n">
         <v>7</v>
-      </c>
-      <c r="K2" t="n">
-        <v>6</v>
       </c>
     </row>
     <row r="3">
@@ -550,13 +550,13 @@
         </is>
       </c>
       <c r="C3" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="D3" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="E3" t="n">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="F3" t="n">
         <v>4</v>
@@ -565,10 +565,10 @@
         <v>2</v>
       </c>
       <c r="H3" s="2" t="n">
-        <v>0.6667</v>
+        <v>0.5714</v>
       </c>
       <c r="I3" s="2" t="n">
-        <v>0.5</v>
+        <v>0.4</v>
       </c>
       <c r="J3" t="n">
         <v>6</v>
@@ -587,13 +587,13 @@
         </is>
       </c>
       <c r="C4" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D4" t="n">
         <v>1</v>
       </c>
       <c r="E4" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="F4" t="n">
         <v>0</v>
@@ -661,13 +661,13 @@
         </is>
       </c>
       <c r="C6" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="D6" t="n">
         <v>4</v>
       </c>
       <c r="E6" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="F6" t="n">
         <v>3</v>
@@ -676,7 +676,7 @@
         <v>1</v>
       </c>
       <c r="H6" s="2" t="n">
-        <v>0.75</v>
+        <v>0.6</v>
       </c>
       <c r="I6" s="2" t="n">
         <v>0.25</v>
@@ -949,13 +949,13 @@
         </is>
       </c>
       <c r="C14" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D14" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="E14" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="F14" t="n">
         <v>0</v>
@@ -967,7 +967,7 @@
         <v>0</v>
       </c>
       <c r="I14" s="2" t="n">
-        <v>0.3333</v>
+        <v>0.25</v>
       </c>
       <c r="J14" t="n">
         <v>1</v>
@@ -986,13 +986,13 @@
         </is>
       </c>
       <c r="C15" t="n">
+        <v>5</v>
+      </c>
+      <c r="D15" t="n">
         <v>4</v>
       </c>
-      <c r="D15" t="n">
-        <v>3</v>
-      </c>
       <c r="E15" t="n">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="F15" t="n">
         <v>2</v>
@@ -1001,7 +1001,7 @@
         <v>0</v>
       </c>
       <c r="H15" s="2" t="n">
-        <v>0.5</v>
+        <v>0.4</v>
       </c>
       <c r="I15" s="2" t="n">
         <v>0</v>
@@ -1315,6 +1315,12 @@
       <c r="L3" t="n">
         <v>1</v>
       </c>
+      <c r="N3" t="n">
+        <v>1</v>
+      </c>
+      <c r="O3" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -1352,6 +1358,12 @@
       <c r="L4" t="n">
         <v>1</v>
       </c>
+      <c r="N4" t="n">
+        <v>0</v>
+      </c>
+      <c r="O4" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -1368,6 +1380,9 @@
       <c r="L5" t="n">
         <v>0</v>
       </c>
+      <c r="N5" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -1421,6 +1436,9 @@
       <c r="I7" t="n">
         <v>0</v>
       </c>
+      <c r="N7" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -1555,6 +1573,12 @@
       <c r="K15" t="n">
         <v>0</v>
       </c>
+      <c r="N15" t="n">
+        <v>0</v>
+      </c>
+      <c r="O15" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -1581,6 +1605,12 @@
         <v>0</v>
       </c>
       <c r="L16" t="n">
+        <v>0</v>
+      </c>
+      <c r="N16" t="n">
+        <v>0</v>
+      </c>
+      <c r="O16" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1630,7 +1660,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H73"/>
+  <dimension ref="A1:H83"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -4560,6 +4590,402 @@
         </is>
       </c>
       <c r="H73" t="inlineStr">
+        <is>
+          <t>L</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="B74" t="inlineStr">
+        <is>
+          <t>21.06.2026</t>
+        </is>
+      </c>
+      <c r="C74" t="inlineStr">
+        <is>
+          <t>TC ESO Praha z.s. A</t>
+        </is>
+      </c>
+      <c r="D74" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="E74" t="inlineStr">
+        <is>
+          <t>singl</t>
+        </is>
+      </c>
+      <c r="F74" t="inlineStr">
+        <is>
+          <t>Tichý Ján</t>
+        </is>
+      </c>
+      <c r="G74" t="inlineStr"/>
+      <c r="H74" t="inlineStr">
+        <is>
+          <t>W</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="B75" t="inlineStr">
+        <is>
+          <t>21.06.2026</t>
+        </is>
+      </c>
+      <c r="C75" t="inlineStr">
+        <is>
+          <t>TC ESO Praha z.s. A</t>
+        </is>
+      </c>
+      <c r="D75" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="E75" t="inlineStr">
+        <is>
+          <t>singl</t>
+        </is>
+      </c>
+      <c r="F75" t="inlineStr">
+        <is>
+          <t>Schwarz Ondřej</t>
+        </is>
+      </c>
+      <c r="G75" t="inlineStr"/>
+      <c r="H75" t="inlineStr">
+        <is>
+          <t>L</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="B76" t="inlineStr">
+        <is>
+          <t>21.06.2026</t>
+        </is>
+      </c>
+      <c r="C76" t="inlineStr">
+        <is>
+          <t>TC ESO Praha z.s. A</t>
+        </is>
+      </c>
+      <c r="D76" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="E76" t="inlineStr">
+        <is>
+          <t>singl</t>
+        </is>
+      </c>
+      <c r="F76" t="inlineStr">
+        <is>
+          <t>Kotlasová Klára</t>
+        </is>
+      </c>
+      <c r="G76" t="inlineStr"/>
+      <c r="H76" t="inlineStr">
+        <is>
+          <t>L</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="B77" t="inlineStr">
+        <is>
+          <t>21.06.2026</t>
+        </is>
+      </c>
+      <c r="C77" t="inlineStr">
+        <is>
+          <t>TC ESO Praha z.s. A</t>
+        </is>
+      </c>
+      <c r="D77" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="E77" t="inlineStr">
+        <is>
+          <t>singl</t>
+        </is>
+      </c>
+      <c r="F77" t="inlineStr">
+        <is>
+          <t>Hádková Anna</t>
+        </is>
+      </c>
+      <c r="G77" t="inlineStr"/>
+      <c r="H77" t="inlineStr">
+        <is>
+          <t>L</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="B78" t="inlineStr">
+        <is>
+          <t>21.06.2026</t>
+        </is>
+      </c>
+      <c r="C78" t="inlineStr">
+        <is>
+          <t>TC ESO Praha z.s. A</t>
+        </is>
+      </c>
+      <c r="D78" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="E78" t="inlineStr">
+        <is>
+          <t>singl</t>
+        </is>
+      </c>
+      <c r="F78" t="inlineStr">
+        <is>
+          <t>Kosík Jan</t>
+        </is>
+      </c>
+      <c r="G78" t="inlineStr"/>
+      <c r="H78" t="inlineStr">
+        <is>
+          <t>L</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="B79" t="inlineStr">
+        <is>
+          <t>21.06.2026</t>
+        </is>
+      </c>
+      <c r="C79" t="inlineStr">
+        <is>
+          <t>TC ESO Praha z.s. A</t>
+        </is>
+      </c>
+      <c r="D79" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="E79" t="inlineStr">
+        <is>
+          <t>singl</t>
+        </is>
+      </c>
+      <c r="F79" t="inlineStr">
+        <is>
+          <t>Motl Ondřej (H)</t>
+        </is>
+      </c>
+      <c r="G79" t="inlineStr"/>
+      <c r="H79" t="inlineStr">
+        <is>
+          <t>L</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="B80" t="inlineStr">
+        <is>
+          <t>21.06.2026</t>
+        </is>
+      </c>
+      <c r="C80" t="inlineStr">
+        <is>
+          <t>TC ESO Praha z.s. A</t>
+        </is>
+      </c>
+      <c r="D80" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="E80" t="inlineStr">
+        <is>
+          <t>debl</t>
+        </is>
+      </c>
+      <c r="F80" t="inlineStr">
+        <is>
+          <t>Kotlasová Klára</t>
+        </is>
+      </c>
+      <c r="G80" t="inlineStr">
+        <is>
+          <t>Hádková Anna</t>
+        </is>
+      </c>
+      <c r="H80" t="inlineStr">
+        <is>
+          <t>L</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="B81" t="inlineStr">
+        <is>
+          <t>21.06.2026</t>
+        </is>
+      </c>
+      <c r="C81" t="inlineStr">
+        <is>
+          <t>TC ESO Praha z.s. A</t>
+        </is>
+      </c>
+      <c r="D81" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="E81" t="inlineStr">
+        <is>
+          <t>debl</t>
+        </is>
+      </c>
+      <c r="F81" t="inlineStr">
+        <is>
+          <t>Hádková Anna</t>
+        </is>
+      </c>
+      <c r="G81" t="inlineStr">
+        <is>
+          <t>Kotlasová Klára</t>
+        </is>
+      </c>
+      <c r="H81" t="inlineStr">
+        <is>
+          <t>L</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="B82" t="inlineStr">
+        <is>
+          <t>21.06.2026</t>
+        </is>
+      </c>
+      <c r="C82" t="inlineStr">
+        <is>
+          <t>TC ESO Praha z.s. A</t>
+        </is>
+      </c>
+      <c r="D82" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
+      <c r="E82" t="inlineStr">
+        <is>
+          <t>debl</t>
+        </is>
+      </c>
+      <c r="F82" t="inlineStr">
+        <is>
+          <t>Tichý Ján</t>
+        </is>
+      </c>
+      <c r="G82" t="inlineStr">
+        <is>
+          <t>Schwarz Ondřej</t>
+        </is>
+      </c>
+      <c r="H82" t="inlineStr">
+        <is>
+          <t>L</t>
+        </is>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="B83" t="inlineStr">
+        <is>
+          <t>21.06.2026</t>
+        </is>
+      </c>
+      <c r="C83" t="inlineStr">
+        <is>
+          <t>TC ESO Praha z.s. A</t>
+        </is>
+      </c>
+      <c r="D83" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
+      <c r="E83" t="inlineStr">
+        <is>
+          <t>debl</t>
+        </is>
+      </c>
+      <c r="F83" t="inlineStr">
+        <is>
+          <t>Schwarz Ondřej</t>
+        </is>
+      </c>
+      <c r="G83" t="inlineStr">
+        <is>
+          <t>Tichý Ján</t>
+        </is>
+      </c>
+      <c r="H83" t="inlineStr">
         <is>
           <t>L</t>
         </is>
@@ -4712,39 +5138,39 @@
         </is>
       </c>
       <c r="C3" t="n">
+        <v>7</v>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>Tichý Ján</t>
+        </is>
+      </c>
+      <c r="E3" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>Kosík Jan</t>
+        </is>
+      </c>
+      <c r="G3" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>Schwarz Ondřej</t>
+        </is>
+      </c>
+      <c r="I3" t="n">
+        <v>12</v>
+      </c>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>Tichý Ján</t>
+        </is>
+      </c>
+      <c r="K3" t="n">
         <v>6</v>
-      </c>
-      <c r="D3" t="inlineStr">
-        <is>
-          <t>Tichý Ján</t>
-        </is>
-      </c>
-      <c r="E3" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="F3" t="inlineStr">
-        <is>
-          <t>Kosík Jan</t>
-        </is>
-      </c>
-      <c r="G3" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="H3" t="inlineStr">
-        <is>
-          <t>Schwarz Ondřej</t>
-        </is>
-      </c>
-      <c r="I3" t="n">
-        <v>10</v>
-      </c>
-      <c r="J3" t="inlineStr">
-        <is>
-          <t>Tichý Ján</t>
-        </is>
-      </c>
-      <c r="K3" t="n">
-        <v>5</v>
       </c>
       <c r="L3" t="inlineStr">
         <is>
@@ -4775,7 +5201,7 @@
         </is>
       </c>
       <c r="E4" s="2" t="n">
-        <v>0.75</v>
+        <v>0.6</v>
       </c>
       <c r="F4" t="inlineStr">
         <is>
@@ -4783,7 +5209,7 @@
         </is>
       </c>
       <c r="G4" s="2" t="n">
-        <v>0.5</v>
+        <v>0.4</v>
       </c>
       <c r="H4" t="inlineStr">
         <is>
@@ -4791,7 +5217,7 @@
         </is>
       </c>
       <c r="I4" t="n">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="J4" t="inlineStr">
         <is>
@@ -4830,7 +5256,7 @@
         </is>
       </c>
       <c r="E5" s="2" t="n">
-        <v>0.6667</v>
+        <v>0.5714</v>
       </c>
       <c r="F5" t="inlineStr">
         <is>
@@ -4838,7 +5264,7 @@
         </is>
       </c>
       <c r="G5" s="2" t="n">
-        <v>0.5</v>
+        <v>0.4</v>
       </c>
       <c r="H5" t="inlineStr">
         <is>
@@ -4846,7 +5272,7 @@
         </is>
       </c>
       <c r="I5" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="J5" t="inlineStr">
         <is>
@@ -4897,11 +5323,11 @@
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>Kučera Denis (H)</t>
+          <t>Hádková Anna</t>
         </is>
       </c>
       <c r="I6" t="n">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="J6" t="inlineStr">
         <is>
@@ -4940,7 +5366,7 @@
         </is>
       </c>
       <c r="E7" s="2" t="n">
-        <v>0.5</v>
+        <v>0.4</v>
       </c>
       <c r="F7" t="inlineStr">
         <is>
@@ -4952,11 +5378,11 @@
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>Skopcová Valerie</t>
+          <t>Kotlasová Klára</t>
         </is>
       </c>
       <c r="I7" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="J7" t="inlineStr">
         <is>
@@ -4999,15 +5425,15 @@
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>Kotlasová Klára</t>
+          <t>Motl Ondřej (H)</t>
         </is>
       </c>
       <c r="G8" s="2" t="n">
-        <v>0.3333</v>
+        <v>0.25</v>
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>Hádková Anna</t>
+          <t>Kučera Denis (H)</t>
         </is>
       </c>
       <c r="I8" t="n">
@@ -5054,7 +5480,7 @@
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>Motl Ondřej (H)</t>
+          <t>Kučera Denis (H)</t>
         </is>
       </c>
       <c r="G9" s="2" t="n">
@@ -5062,11 +5488,11 @@
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>Kotlasová Klára</t>
+          <t>Skopcová Valerie</t>
         </is>
       </c>
       <c r="I9" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="J9" t="inlineStr">
         <is>
@@ -5109,7 +5535,7 @@
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>Kučera Denis (H)</t>
+          <t>Kotlasová Klára</t>
         </is>
       </c>
       <c r="G10" s="2" t="n">
@@ -5176,7 +5602,7 @@
         </is>
       </c>
       <c r="I11" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="J11" t="inlineStr">
         <is>

</xml_diff>